<commit_message>
código para la memoria
</commit_message>
<xml_diff>
--- a/Resultados.xlsx
+++ b/Resultados.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alvar\Desktop\TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBD10E5-239E-4FFD-8B33-236124FB62B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979A0CD3-2EC7-497C-8E95-6ADBC512F4D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Final" sheetId="3" r:id="rId1"/>
@@ -1184,6 +1184,243 @@
     <xf numFmtId="10" fontId="2" fillId="7" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="49" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="40" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="42" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="45" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="43" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="2" borderId="50" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="2" borderId="51" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="2" borderId="52" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="39" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="27" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="28" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="28" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="29" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="21" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="30" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="25" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="35" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="20" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="21" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="10" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="32" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1193,15 +1430,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1210,234 +1438,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="30" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="25" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="35" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="20" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="21" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="10" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="21" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="32" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="28" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="27" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="28" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="29" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="47" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="48" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="49" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="40" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="42" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="45" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="6" borderId="43" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="2" borderId="50" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="2" borderId="51" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="2" borderId="52" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="39" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1740,6 +1740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9F9982B-AEC3-4290-84FC-3F89627A1106}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="B1:Q21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1759,38 +1760,38 @@
   <sheetData>
     <row r="1" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="59" t="s">
+      <c r="D2" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="59" t="s">
+      <c r="E2" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="59" t="s">
+      <c r="F2" s="99" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
+      <c r="G2" s="99"/>
+      <c r="H2" s="99"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="99"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="99"/>
+      <c r="N2" s="99"/>
+      <c r="O2" s="99"/>
       <c r="P2" s="27"/>
       <c r="Q2" s="27"/>
     </row>
     <row r="3" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="59"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
       <c r="F3" s="41" t="s">
         <v>2</v>
       </c>
@@ -1825,16 +1826,16 @@
       <c r="Q3" s="23"/>
     </row>
     <row r="4" spans="2:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="75" t="s">
+      <c r="C4" s="110" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="77">
+      <c r="D4" s="112">
         <v>0.23810000000000001</v>
       </c>
-      <c r="E4" s="79">
+      <c r="E4" s="114">
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="F4" s="35">
@@ -1871,10 +1872,10 @@
       <c r="Q4" s="26"/>
     </row>
     <row r="5" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="64"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="78"/>
-      <c r="E5" s="80"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="115"/>
       <c r="F5" s="32">
         <v>0.107</v>
       </c>
@@ -1909,14 +1910,14 @@
       <c r="Q5" s="26"/>
     </row>
     <row r="6" spans="2:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="64"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="72"/>
+      <c r="C6" s="116" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="77">
+      <c r="D6" s="112">
         <v>0.2296</v>
       </c>
-      <c r="E6" s="79">
+      <c r="E6" s="114">
         <v>3.6400000000000002E-2</v>
       </c>
       <c r="F6" s="35">
@@ -1953,10 +1954,10 @@
       <c r="Q6" s="26"/>
     </row>
     <row r="7" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="64"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="78"/>
-      <c r="E7" s="80"/>
+      <c r="B7" s="72"/>
+      <c r="C7" s="117"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="115"/>
       <c r="F7" s="32">
         <v>0.1096</v>
       </c>
@@ -1991,16 +1992,16 @@
       <c r="Q7" s="26"/>
     </row>
     <row r="8" spans="2:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="66" t="s">
+      <c r="B8" s="118" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="69" t="s">
+      <c r="C8" s="121" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="125">
         <v>0.33479999999999999</v>
       </c>
-      <c r="E8" s="71">
+      <c r="E8" s="123">
         <v>3.7400000000000003E-2</v>
       </c>
       <c r="F8" s="38">
@@ -2037,10 +2038,10 @@
       <c r="Q8" s="25"/>
     </row>
     <row r="9" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="67"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="72"/>
+      <c r="B9" s="119"/>
+      <c r="C9" s="122"/>
+      <c r="D9" s="126"/>
+      <c r="E9" s="124"/>
       <c r="F9" s="29">
         <v>8.2299999999999998E-2</v>
       </c>
@@ -2075,14 +2076,14 @@
       <c r="Q9" s="25"/>
     </row>
     <row r="10" spans="2:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="67"/>
-      <c r="C10" s="81" t="s">
+      <c r="B10" s="119"/>
+      <c r="C10" s="127" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="73">
+      <c r="D10" s="125">
         <v>0.34399999999999997</v>
       </c>
-      <c r="E10" s="71">
+      <c r="E10" s="123">
         <v>4.0500000000000001E-2</v>
       </c>
       <c r="F10" s="38">
@@ -2119,10 +2120,10 @@
       <c r="Q10" s="25"/>
     </row>
     <row r="11" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="68"/>
-      <c r="C11" s="82"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="72"/>
+      <c r="B11" s="120"/>
+      <c r="C11" s="128"/>
+      <c r="D11" s="126"/>
+      <c r="E11" s="124"/>
       <c r="F11" s="29">
         <v>9.5600000000000004E-2</v>
       </c>
@@ -2157,11 +2158,11 @@
       <c r="Q11" s="25"/>
     </row>
     <row r="12" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="60" t="s">
+      <c r="C12" s="74" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="61"/>
-      <c r="E12" s="62"/>
+      <c r="D12" s="75"/>
+      <c r="E12" s="76"/>
       <c r="F12" s="13">
         <v>0.59499999999999997</v>
       </c>
@@ -2194,11 +2195,11 @@
       </c>
     </row>
     <row r="13" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="53" t="s">
+      <c r="C13" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="54"/>
-      <c r="E13" s="55"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="79"/>
       <c r="F13" s="19">
         <v>0.39357755999999999</v>
       </c>
@@ -2231,11 +2232,11 @@
       </c>
     </row>
     <row r="14" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="54"/>
-      <c r="E14" s="55"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="79"/>
       <c r="F14" s="44">
         <v>0.63429999999999997</v>
       </c>
@@ -2270,11 +2271,11 @@
       <c r="Q14" s="25"/>
     </row>
     <row r="15" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="56" t="s">
+      <c r="C15" s="132" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="57"/>
-      <c r="E15" s="58"/>
+      <c r="D15" s="133"/>
+      <c r="E15" s="134"/>
       <c r="F15" s="47">
         <v>0.75190000000000001</v>
       </c>
@@ -2310,11 +2311,11 @@
     </row>
     <row r="16" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="28"/>
-      <c r="C16" s="50" t="s">
+      <c r="C16" s="129" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="51"/>
-      <c r="E16" s="52"/>
+      <c r="D16" s="130"/>
+      <c r="E16" s="131"/>
       <c r="F16" s="47">
         <v>0.52395343999999999</v>
       </c>
@@ -2350,11 +2351,11 @@
     </row>
     <row r="17" spans="2:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="28"/>
-      <c r="C17" s="50" t="s">
+      <c r="C17" s="129" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="51"/>
-      <c r="E17" s="52"/>
+      <c r="D17" s="130"/>
+      <c r="E17" s="131"/>
       <c r="F17" s="47">
         <v>0.69679999999999997</v>
       </c>
@@ -2435,10 +2436,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
     <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="F2:O2"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B4:B7"/>
@@ -2446,20 +2452,15 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="E8:E9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2467,6 +2468,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{186B5B65-350C-4C08-9EDC-FA7F49A76224}">
+  <sheetPr codeName="Hoja3"/>
   <dimension ref="B1:L25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2483,803 +2485,803 @@
   <sheetData>
     <row r="1" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="114" t="s">
+      <c r="B2" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="115" t="s">
+      <c r="C2" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="116" t="s">
+      <c r="D2" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="116" t="s">
+      <c r="E2" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="116" t="s">
+      <c r="F2" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="116" t="s">
+      <c r="G2" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="116" t="s">
+      <c r="H2" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="116" t="s">
+      <c r="I2" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="116" t="s">
+      <c r="J2" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="116" t="s">
+      <c r="K2" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="117" t="s">
+      <c r="L2" s="53" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="133" t="s">
+      <c r="C3" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="122">
+      <c r="D3" s="58">
         <v>0.03</v>
       </c>
-      <c r="E3" s="122">
+      <c r="E3" s="58">
         <v>0.12</v>
       </c>
-      <c r="F3" s="122">
+      <c r="F3" s="58">
         <v>0.39</v>
       </c>
-      <c r="G3" s="122">
+      <c r="G3" s="58">
         <v>0.1</v>
       </c>
-      <c r="H3" s="122">
+      <c r="H3" s="58">
         <v>0.01</v>
       </c>
-      <c r="I3" s="122">
+      <c r="I3" s="58">
         <v>0.28000000000000003</v>
       </c>
-      <c r="J3" s="122">
+      <c r="J3" s="58">
         <v>0.04</v>
       </c>
-      <c r="K3" s="122">
+      <c r="K3" s="58">
         <v>0.02</v>
       </c>
-      <c r="L3" s="123">
+      <c r="L3" s="59">
         <v>0.01</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="119" t="s">
+      <c r="B4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="124">
+      <c r="C4" s="60">
         <v>0.04</v>
       </c>
-      <c r="D4" s="133" t="s">
+      <c r="D4" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="125">
+      <c r="E4" s="61">
         <v>0.04</v>
       </c>
-      <c r="F4" s="125">
+      <c r="F4" s="61">
         <v>0.43</v>
       </c>
-      <c r="G4" s="125">
+      <c r="G4" s="61">
         <v>0.04</v>
       </c>
-      <c r="H4" s="125">
+      <c r="H4" s="61">
         <v>0.01</v>
       </c>
-      <c r="I4" s="125">
+      <c r="I4" s="61">
         <v>0.39</v>
       </c>
-      <c r="J4" s="125">
+      <c r="J4" s="61">
         <v>0.02</v>
       </c>
-      <c r="K4" s="125">
+      <c r="K4" s="61">
         <v>0.02</v>
       </c>
-      <c r="L4" s="126">
+      <c r="L4" s="62">
         <v>0.02</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="119" t="s">
+      <c r="B5" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="124">
+      <c r="C5" s="60">
         <v>0.35</v>
       </c>
-      <c r="D5" s="125">
+      <c r="D5" s="61">
         <v>0.03</v>
       </c>
-      <c r="E5" s="133" t="s">
+      <c r="E5" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="125">
+      <c r="F5" s="61">
         <v>0.23</v>
       </c>
-      <c r="G5" s="125">
+      <c r="G5" s="61">
         <v>0.03</v>
       </c>
-      <c r="H5" s="125">
+      <c r="H5" s="61">
         <v>0.01</v>
       </c>
-      <c r="I5" s="125">
+      <c r="I5" s="61">
         <v>0.25</v>
       </c>
-      <c r="J5" s="125">
+      <c r="J5" s="61">
         <v>0.02</v>
       </c>
-      <c r="K5" s="125">
+      <c r="K5" s="61">
         <v>0.08</v>
       </c>
-      <c r="L5" s="126">
+      <c r="L5" s="62">
         <v>0.01</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="119" t="s">
+      <c r="B6" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="124">
+      <c r="C6" s="60">
         <v>0.2</v>
       </c>
-      <c r="D6" s="125">
+      <c r="D6" s="61">
         <v>0.03</v>
       </c>
-      <c r="E6" s="125">
+      <c r="E6" s="61">
         <v>0.08</v>
       </c>
-      <c r="F6" s="133" t="s">
+      <c r="F6" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="125">
+      <c r="G6" s="61">
         <v>0.43</v>
       </c>
-      <c r="H6" s="125">
+      <c r="H6" s="61">
         <v>0.03</v>
       </c>
-      <c r="I6" s="125">
+      <c r="I6" s="61">
         <v>0.13</v>
       </c>
-      <c r="J6" s="125">
+      <c r="J6" s="61">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="K6" s="125">
+      <c r="K6" s="61">
         <v>0.02</v>
       </c>
-      <c r="L6" s="126">
+      <c r="L6" s="62">
         <v>0.02</v>
       </c>
     </row>
     <row r="7" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="119" t="s">
+      <c r="B7" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="124">
+      <c r="C7" s="60">
         <v>0.06</v>
       </c>
-      <c r="D7" s="125">
+      <c r="D7" s="61">
         <v>0.01</v>
       </c>
-      <c r="E7" s="125">
+      <c r="E7" s="61">
         <v>0.01</v>
       </c>
-      <c r="F7" s="125">
+      <c r="F7" s="61">
         <v>0.82</v>
       </c>
-      <c r="G7" s="133" t="s">
+      <c r="G7" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="125">
+      <c r="H7" s="61">
         <v>0.01</v>
       </c>
-      <c r="I7" s="125">
+      <c r="I7" s="61">
         <v>0.06</v>
       </c>
-      <c r="J7" s="125">
+      <c r="J7" s="61">
         <v>0.01</v>
       </c>
-      <c r="K7" s="125">
+      <c r="K7" s="61">
         <v>0.01</v>
       </c>
-      <c r="L7" s="126">
+      <c r="L7" s="62">
         <v>0.02</v>
       </c>
     </row>
     <row r="8" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="119" t="s">
+      <c r="B8" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="124">
+      <c r="C8" s="60">
         <v>0.04</v>
       </c>
-      <c r="D8" s="125">
+      <c r="D8" s="61">
         <v>0.02</v>
       </c>
-      <c r="E8" s="125">
+      <c r="E8" s="61">
         <v>0.02</v>
       </c>
-      <c r="F8" s="125">
+      <c r="F8" s="61">
         <v>0.45</v>
       </c>
-      <c r="G8" s="125">
+      <c r="G8" s="61">
         <v>0.03</v>
       </c>
-      <c r="H8" s="133" t="s">
+      <c r="H8" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="125">
+      <c r="I8" s="61">
         <v>0.3</v>
       </c>
-      <c r="J8" s="125">
+      <c r="J8" s="61">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="K8" s="125">
+      <c r="K8" s="61">
         <v>0.03</v>
       </c>
-      <c r="L8" s="126">
+      <c r="L8" s="62">
         <v>0.03</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="119" t="s">
+      <c r="B9" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="124">
+      <c r="C9" s="60">
         <v>0.26</v>
       </c>
-      <c r="D9" s="125">
+      <c r="D9" s="61">
         <v>0.01</v>
       </c>
-      <c r="E9" s="125">
+      <c r="E9" s="61">
         <v>0.06</v>
       </c>
-      <c r="F9" s="125">
+      <c r="F9" s="61">
         <v>0.48</v>
       </c>
-      <c r="G9" s="125">
+      <c r="G9" s="61">
         <v>0.05</v>
       </c>
-      <c r="H9" s="125">
+      <c r="H9" s="61">
         <v>0.03</v>
       </c>
-      <c r="I9" s="133" t="s">
+      <c r="I9" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="125">
+      <c r="J9" s="61">
         <v>0.08</v>
       </c>
-      <c r="K9" s="125">
+      <c r="K9" s="61">
         <v>0.02</v>
       </c>
-      <c r="L9" s="126">
+      <c r="L9" s="62">
         <v>0.02</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="119" t="s">
+      <c r="B10" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="124">
+      <c r="C10" s="60">
         <v>0.1</v>
       </c>
-      <c r="D10" s="125">
+      <c r="D10" s="61">
         <v>0.06</v>
       </c>
-      <c r="E10" s="125">
+      <c r="E10" s="61">
         <v>0.26</v>
       </c>
-      <c r="F10" s="125">
+      <c r="F10" s="61">
         <v>0.31</v>
       </c>
-      <c r="G10" s="125">
+      <c r="G10" s="61">
         <v>0.03</v>
       </c>
-      <c r="H10" s="125">
+      <c r="H10" s="61">
         <v>0.02</v>
       </c>
-      <c r="I10" s="125">
+      <c r="I10" s="61">
         <v>0.14000000000000001</v>
       </c>
-      <c r="J10" s="133" t="s">
+      <c r="J10" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="125">
+      <c r="K10" s="61">
         <v>0.05</v>
       </c>
-      <c r="L10" s="126">
+      <c r="L10" s="62">
         <v>0.03</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="119" t="s">
+      <c r="B11" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="124">
+      <c r="C11" s="60">
         <v>0.02</v>
       </c>
-      <c r="D11" s="125">
+      <c r="D11" s="61">
         <v>0.03</v>
       </c>
-      <c r="E11" s="125">
+      <c r="E11" s="61">
         <v>0.02</v>
       </c>
-      <c r="F11" s="125">
+      <c r="F11" s="61">
         <v>0.8</v>
       </c>
-      <c r="G11" s="125">
+      <c r="G11" s="61">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="H11" s="125">
+      <c r="H11" s="61">
         <v>0.01</v>
       </c>
-      <c r="I11" s="125">
+      <c r="I11" s="61">
         <v>0.01</v>
       </c>
-      <c r="J11" s="125">
+      <c r="J11" s="61">
         <v>0.02</v>
       </c>
-      <c r="K11" s="133" t="s">
+      <c r="K11" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="126">
+      <c r="L11" s="62">
         <v>0.01</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="120" t="s">
+      <c r="B12" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="127">
+      <c r="C12" s="63">
         <v>0.01</v>
       </c>
-      <c r="D12" s="128">
+      <c r="D12" s="64">
         <v>0.02</v>
       </c>
-      <c r="E12" s="128">
+      <c r="E12" s="64">
         <v>0</v>
       </c>
-      <c r="F12" s="128">
+      <c r="F12" s="64">
         <v>0.72</v>
       </c>
-      <c r="G12" s="128">
+      <c r="G12" s="64">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="H12" s="128">
+      <c r="H12" s="64">
         <v>0.02</v>
       </c>
-      <c r="I12" s="128">
+      <c r="I12" s="64">
         <v>0.11</v>
       </c>
-      <c r="J12" s="128">
+      <c r="J12" s="64">
         <v>0.05</v>
       </c>
-      <c r="K12" s="128">
+      <c r="K12" s="64">
         <v>0.01</v>
       </c>
-      <c r="L12" s="134" t="s">
+      <c r="L12" s="70" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="121"/>
-      <c r="C13" s="129"/>
-      <c r="D13" s="129"/>
-      <c r="E13" s="129"/>
-      <c r="F13" s="129"/>
-      <c r="G13" s="129"/>
-      <c r="H13" s="129"/>
-      <c r="I13" s="129"/>
-      <c r="J13" s="129"/>
-      <c r="K13" s="129"/>
-      <c r="L13" s="129"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="65"/>
+      <c r="F13" s="65"/>
+      <c r="G13" s="65"/>
+      <c r="H13" s="65"/>
+      <c r="I13" s="65"/>
+      <c r="J13" s="65"/>
+      <c r="K13" s="65"/>
+      <c r="L13" s="65"/>
     </row>
     <row r="14" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="121"/>
-      <c r="C14" s="129"/>
-      <c r="D14" s="129"/>
-      <c r="E14" s="129"/>
-      <c r="F14" s="129"/>
-      <c r="G14" s="129"/>
-      <c r="H14" s="129"/>
-      <c r="I14" s="129"/>
-      <c r="J14" s="129"/>
-      <c r="K14" s="129"/>
-      <c r="L14" s="129"/>
+      <c r="B14" s="57"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="65"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="65"/>
     </row>
     <row r="15" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="114" t="s">
+      <c r="B15" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="130" t="s">
+      <c r="C15" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="131" t="s">
+      <c r="D15" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="131" t="s">
+      <c r="E15" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="131" t="s">
+      <c r="F15" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="131" t="s">
+      <c r="G15" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="H15" s="131" t="s">
+      <c r="H15" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="I15" s="131" t="s">
+      <c r="I15" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="J15" s="131" t="s">
+      <c r="J15" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="K15" s="131" t="s">
+      <c r="K15" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="L15" s="132" t="s">
+      <c r="L15" s="68" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="118" t="s">
+      <c r="B16" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="133" t="s">
+      <c r="C16" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="122">
+      <c r="D16" s="58">
         <v>0.09</v>
       </c>
-      <c r="E16" s="122">
+      <c r="E16" s="58">
         <v>0.05</v>
       </c>
-      <c r="F16" s="122">
+      <c r="F16" s="58">
         <v>0.33</v>
       </c>
-      <c r="G16" s="122">
+      <c r="G16" s="58">
         <v>0.05</v>
       </c>
-      <c r="H16" s="122">
+      <c r="H16" s="58">
         <v>0.03</v>
       </c>
-      <c r="I16" s="122">
+      <c r="I16" s="58">
         <v>0.35</v>
       </c>
-      <c r="J16" s="122">
+      <c r="J16" s="58">
         <v>0.05</v>
       </c>
-      <c r="K16" s="122">
+      <c r="K16" s="58">
         <v>0.02</v>
       </c>
-      <c r="L16" s="123">
+      <c r="L16" s="59">
         <v>0.04</v>
       </c>
     </row>
     <row r="17" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="119" t="s">
+      <c r="B17" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="C17" s="124">
+      <c r="C17" s="60">
         <v>0.66</v>
       </c>
-      <c r="D17" s="133" t="s">
+      <c r="D17" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="125">
+      <c r="E17" s="61">
         <v>0.01</v>
       </c>
-      <c r="F17" s="125">
+      <c r="F17" s="61">
         <v>0.16</v>
       </c>
-      <c r="G17" s="125">
+      <c r="G17" s="61">
         <v>0.01</v>
       </c>
-      <c r="H17" s="125">
+      <c r="H17" s="61">
         <v>0.01</v>
       </c>
-      <c r="I17" s="125">
+      <c r="I17" s="61">
         <v>0.09</v>
       </c>
-      <c r="J17" s="125">
+      <c r="J17" s="61">
         <v>0.02</v>
       </c>
-      <c r="K17" s="125">
+      <c r="K17" s="61">
         <v>0.01</v>
       </c>
-      <c r="L17" s="126">
+      <c r="L17" s="62">
         <v>0.03</v>
       </c>
     </row>
     <row r="18" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="119" t="s">
+      <c r="B18" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="124">
+      <c r="C18" s="60">
         <v>0.41</v>
       </c>
-      <c r="D18" s="125">
+      <c r="D18" s="61">
         <v>0.36</v>
       </c>
-      <c r="E18" s="133" t="s">
+      <c r="E18" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="F18" s="125">
+      <c r="F18" s="61">
         <v>0</v>
       </c>
-      <c r="G18" s="125">
+      <c r="G18" s="61">
         <v>0.01</v>
       </c>
-      <c r="H18" s="125">
+      <c r="H18" s="61">
         <v>0.04</v>
       </c>
-      <c r="I18" s="125">
+      <c r="I18" s="61">
         <v>0</v>
       </c>
-      <c r="J18" s="125">
+      <c r="J18" s="61">
         <v>0</v>
       </c>
-      <c r="K18" s="125">
+      <c r="K18" s="61">
         <v>0.1</v>
       </c>
-      <c r="L18" s="126">
+      <c r="L18" s="62">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="19" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="119" t="s">
+      <c r="B19" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="124">
+      <c r="C19" s="60">
         <v>0.5</v>
       </c>
-      <c r="D19" s="125">
+      <c r="D19" s="61">
         <v>0.05</v>
       </c>
-      <c r="E19" s="125">
+      <c r="E19" s="61">
         <v>0.03</v>
       </c>
-      <c r="F19" s="133" t="s">
+      <c r="F19" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="125">
+      <c r="G19" s="61">
         <v>0.06</v>
       </c>
-      <c r="H19" s="125">
+      <c r="H19" s="61">
         <v>0.03</v>
       </c>
-      <c r="I19" s="125">
+      <c r="I19" s="61">
         <v>0.24</v>
       </c>
-      <c r="J19" s="125">
+      <c r="J19" s="61">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="K19" s="125">
+      <c r="K19" s="61">
         <v>0.02</v>
       </c>
-      <c r="L19" s="126">
+      <c r="L19" s="62">
         <v>0.01</v>
       </c>
     </row>
     <row r="20" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="119" t="s">
+      <c r="B20" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="124">
+      <c r="C20" s="60">
         <v>0.34</v>
       </c>
-      <c r="D20" s="125">
+      <c r="D20" s="61">
         <v>0.01</v>
       </c>
-      <c r="E20" s="125">
+      <c r="E20" s="61">
         <v>0.02</v>
       </c>
-      <c r="F20" s="125">
+      <c r="F20" s="61">
         <v>0.43</v>
       </c>
-      <c r="G20" s="133" t="s">
+      <c r="G20" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="125">
+      <c r="H20" s="61">
         <v>0.01</v>
       </c>
-      <c r="I20" s="125">
+      <c r="I20" s="61">
         <v>0.13</v>
       </c>
-      <c r="J20" s="125">
+      <c r="J20" s="61">
         <v>0.02</v>
       </c>
-      <c r="K20" s="125">
+      <c r="K20" s="61">
         <v>0.01</v>
       </c>
-      <c r="L20" s="126">
+      <c r="L20" s="62">
         <v>0.03</v>
       </c>
     </row>
     <row r="21" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="119" t="s">
+      <c r="B21" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="124">
+      <c r="C21" s="60">
         <v>0.05</v>
       </c>
-      <c r="D21" s="125">
+      <c r="D21" s="61">
         <v>0.18</v>
       </c>
-      <c r="E21" s="125">
+      <c r="E21" s="61">
         <v>0.1</v>
       </c>
-      <c r="F21" s="125">
+      <c r="F21" s="61">
         <v>0.19</v>
       </c>
-      <c r="G21" s="125">
+      <c r="G21" s="61">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="H21" s="133" t="s">
+      <c r="H21" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="125">
+      <c r="I21" s="61">
         <v>0</v>
       </c>
-      <c r="J21" s="125">
+      <c r="J21" s="61">
         <v>0.08</v>
       </c>
-      <c r="K21" s="125">
+      <c r="K21" s="61">
         <v>0.11</v>
       </c>
-      <c r="L21" s="126">
+      <c r="L21" s="62">
         <v>0.23</v>
       </c>
     </row>
     <row r="22" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="119" t="s">
+      <c r="B22" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="124">
+      <c r="C22" s="60">
         <v>0.66</v>
       </c>
-      <c r="D22" s="125">
+      <c r="D22" s="61">
         <v>0.03</v>
       </c>
-      <c r="E22" s="125">
+      <c r="E22" s="61">
         <v>0.02</v>
       </c>
-      <c r="F22" s="125">
+      <c r="F22" s="61">
         <v>0.13</v>
       </c>
-      <c r="G22" s="125">
+      <c r="G22" s="61">
         <v>0.02</v>
       </c>
-      <c r="H22" s="125">
+      <c r="H22" s="61">
         <v>0.04</v>
       </c>
-      <c r="I22" s="133" t="s">
+      <c r="I22" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="J22" s="125">
+      <c r="J22" s="61">
         <v>0.03</v>
       </c>
-      <c r="K22" s="125">
+      <c r="K22" s="61">
         <v>0.03</v>
       </c>
-      <c r="L22" s="126">
+      <c r="L22" s="62">
         <v>0.04</v>
       </c>
     </row>
     <row r="23" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="119" t="s">
+      <c r="B23" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="124">
+      <c r="C23" s="60">
         <v>0.1</v>
       </c>
-      <c r="D23" s="125">
+      <c r="D23" s="61">
         <v>0.02</v>
       </c>
-      <c r="E23" s="125">
+      <c r="E23" s="61">
         <v>0.01</v>
       </c>
-      <c r="F23" s="125">
+      <c r="F23" s="61">
         <v>0.57999999999999996</v>
       </c>
-      <c r="G23" s="125">
+      <c r="G23" s="61">
         <v>0.02</v>
       </c>
-      <c r="H23" s="125">
+      <c r="H23" s="61">
         <v>0.02</v>
       </c>
-      <c r="I23" s="125">
+      <c r="I23" s="61">
         <v>0.23</v>
       </c>
-      <c r="J23" s="133" t="s">
+      <c r="J23" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="K23" s="125">
+      <c r="K23" s="61">
         <v>0.02</v>
       </c>
-      <c r="L23" s="126">
+      <c r="L23" s="62">
         <v>0.01</v>
       </c>
     </row>
     <row r="24" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="119" t="s">
+      <c r="B24" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="124">
+      <c r="C24" s="60">
         <v>0.4</v>
       </c>
-      <c r="D24" s="125">
+      <c r="D24" s="61">
         <v>0.06</v>
       </c>
-      <c r="E24" s="125">
+      <c r="E24" s="61">
         <v>0.02</v>
       </c>
-      <c r="F24" s="125">
+      <c r="F24" s="61">
         <v>0.33</v>
       </c>
-      <c r="G24" s="125">
+      <c r="G24" s="61">
         <v>0</v>
       </c>
-      <c r="H24" s="125">
+      <c r="H24" s="61">
         <v>0</v>
       </c>
-      <c r="I24" s="125">
+      <c r="I24" s="61">
         <v>0.15</v>
       </c>
-      <c r="J24" s="125">
+      <c r="J24" s="61">
         <v>0.01</v>
       </c>
-      <c r="K24" s="133" t="s">
+      <c r="K24" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="L24" s="126">
+      <c r="L24" s="62">
         <v>0.02</v>
       </c>
     </row>
     <row r="25" spans="2:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="120" t="s">
+      <c r="B25" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="127">
+      <c r="C25" s="63">
         <v>0.41</v>
       </c>
-      <c r="D25" s="128">
+      <c r="D25" s="64">
         <v>0.02</v>
       </c>
-      <c r="E25" s="128">
+      <c r="E25" s="64">
         <v>0.02</v>
       </c>
-      <c r="F25" s="128">
+      <c r="F25" s="64">
         <v>0.27</v>
       </c>
-      <c r="G25" s="128">
+      <c r="G25" s="64">
         <v>0.03</v>
       </c>
-      <c r="H25" s="128">
+      <c r="H25" s="64">
         <v>0.02</v>
       </c>
-      <c r="I25" s="128">
+      <c r="I25" s="64">
         <v>0.18</v>
       </c>
-      <c r="J25" s="128">
+      <c r="J25" s="64">
         <v>0.04</v>
       </c>
-      <c r="K25" s="128">
+      <c r="K25" s="64">
         <v>0.01</v>
       </c>
-      <c r="L25" s="134" t="s">
+      <c r="L25" s="70" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D3:L3 C25:K25 C24:J24 L24 C23:I23 K23:L23 C22:H22 J22:L22 C21:G21 I21:L21 C20:F20 H20:L20 C19:E19 G19:L19 C18:D18 F18:L18 C17 E17:L17 D16:L16 C13:L14 C12:K12 C11:J11 L11 C10:I10 K10:L10 C9:H9 J9:L9 C8:G8 I8:L8 C7:F7 H7:L7 C6:E6 G6:L6 C5:D5 F5:L5 C4 E4:L4">
+  <conditionalFormatting sqref="D3:L3 C4 E4:L4 C5:D5 F5:L5 C6:E6 G6:L6 C7:F7 H7:L7 C8:G8 I8:L8 C9:H9 J9:L9 C10:I10 K10:L10 C11:J11 L11 C12:K12 C13:L14 D16:L16 C17 E17:L17 C18:D18 F18:L18 C19:E19 G19:L19 C20:F20 H20:L20 C21:G21 I21:L21 C22:H22 J22:L22 C23:I23 K23:L23 C24:J24 L24 C25:K25">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>0.19</formula>
     </cfRule>
@@ -3291,6 +3293,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Hoja4"/>
   <dimension ref="B1:Z38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3316,41 +3319,41 @@
   <sheetData>
     <row r="1" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="59" t="s">
+      <c r="D2" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="59" t="s">
+      <c r="E2" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="59" t="s">
+      <c r="F2" s="99" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59" t="s">
+      <c r="G2" s="99"/>
+      <c r="H2" s="99"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="99"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="99"/>
+      <c r="M2" s="99"/>
+      <c r="N2" s="99"/>
+      <c r="O2" s="99"/>
+      <c r="P2" s="99" t="s">
         <v>35</v>
       </c>
-      <c r="Q2" s="59"/>
+      <c r="Q2" s="99"/>
       <c r="R2" s="1"/>
     </row>
     <row r="3" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="59"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
       <c r="F3" s="41" t="s">
         <v>2</v>
       </c>
@@ -3390,16 +3393,16 @@
       <c r="S3" s="2"/>
     </row>
     <row r="4" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="100" t="s">
+      <c r="B4" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="96" t="s">
+      <c r="C4" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="97" t="s">
+      <c r="D4" s="103" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="91">
+      <c r="E4" s="80">
         <v>0.1</v>
       </c>
       <c r="F4" s="11">
@@ -3432,10 +3435,10 @@
       <c r="O4" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="P4" s="89" t="s">
+      <c r="P4" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="Q4" s="88" t="s">
+      <c r="Q4" s="105" t="s">
         <v>19</v>
       </c>
       <c r="S4" s="3" t="s">
@@ -3443,10 +3446,10 @@
       </c>
     </row>
     <row r="5" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="100"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="85"/>
-      <c r="E5" s="92"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="86"/>
+      <c r="D5" s="104"/>
+      <c r="E5" s="81"/>
       <c r="F5" s="12">
         <v>0.63429999999999997</v>
       </c>
@@ -3477,23 +3480,23 @@
       <c r="O5" s="9">
         <v>0.214</v>
       </c>
-      <c r="P5" s="90"/>
-      <c r="Q5" s="87"/>
+      <c r="P5" s="108"/>
+      <c r="Q5" s="106"/>
       <c r="S5" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" spans="2:22" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="95" t="s">
+      <c r="B6" s="102" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="96" t="s">
+      <c r="C6" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="98">
+      <c r="D6" s="89">
         <v>1.1000000000000001</v>
       </c>
-      <c r="E6" s="91">
+      <c r="E6" s="80">
         <v>0.1208</v>
       </c>
       <c r="F6" s="11">
@@ -3526,10 +3529,10 @@
       <c r="O6" s="7">
         <v>5.7999999999999996E-3</v>
       </c>
-      <c r="P6" s="89" t="s">
+      <c r="P6" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="Q6" s="88" t="s">
+      <c r="Q6" s="105" t="s">
         <v>19</v>
       </c>
       <c r="S6" s="5" t="s">
@@ -3537,10 +3540,10 @@
       </c>
     </row>
     <row r="7" spans="2:22" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="95"/>
-      <c r="C7" s="96"/>
-      <c r="D7" s="99"/>
-      <c r="E7" s="92"/>
+      <c r="B7" s="102"/>
+      <c r="C7" s="86"/>
+      <c r="D7" s="90"/>
+      <c r="E7" s="81"/>
       <c r="F7" s="12">
         <v>0.35520000000000002</v>
       </c>
@@ -3571,23 +3574,23 @@
       <c r="O7" s="9">
         <v>0.2117</v>
       </c>
-      <c r="P7" s="90"/>
-      <c r="Q7" s="87"/>
+      <c r="P7" s="108"/>
+      <c r="Q7" s="106"/>
       <c r="S7" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="108" t="s">
+      <c r="B8" s="91" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="111" t="s">
+      <c r="C8" s="96" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="98">
+      <c r="D8" s="89">
         <v>0.3226</v>
       </c>
-      <c r="E8" s="91">
+      <c r="E8" s="80">
         <v>4.3900000000000002E-2</v>
       </c>
       <c r="F8" s="11">
@@ -3620,10 +3623,10 @@
       <c r="O8" s="7">
         <v>1.3599999999999999E-2</v>
       </c>
-      <c r="P8" s="89" t="s">
+      <c r="P8" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="Q8" s="88" t="s">
+      <c r="Q8" s="105" t="s">
         <v>19</v>
       </c>
       <c r="S8" s="6" t="s">
@@ -3631,34 +3634,34 @@
       </c>
     </row>
     <row r="9" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="109"/>
-      <c r="C9" s="102"/>
-      <c r="D9" s="99"/>
-      <c r="E9" s="92"/>
-      <c r="F9" s="85" t="s">
+      <c r="B9" s="92"/>
+      <c r="C9" s="94"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="104" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="86"/>
-      <c r="H9" s="86"/>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
-      <c r="K9" s="86"/>
-      <c r="L9" s="86"/>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="87"/>
-      <c r="P9" s="90"/>
-      <c r="Q9" s="87"/>
+      <c r="G9" s="109"/>
+      <c r="H9" s="109"/>
+      <c r="I9" s="109"/>
+      <c r="J9" s="109"/>
+      <c r="K9" s="109"/>
+      <c r="L9" s="109"/>
+      <c r="M9" s="109"/>
+      <c r="N9" s="109"/>
+      <c r="O9" s="106"/>
+      <c r="P9" s="108"/>
+      <c r="Q9" s="106"/>
     </row>
     <row r="10" spans="2:22" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="109"/>
-      <c r="C10" s="102" t="s">
+      <c r="B10" s="92"/>
+      <c r="C10" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="98">
+      <c r="D10" s="89">
         <v>0.23699999999999999</v>
       </c>
-      <c r="E10" s="91">
+      <c r="E10" s="80">
         <v>3.4099999999999998E-2</v>
       </c>
       <c r="F10" s="11">
@@ -3691,44 +3694,44 @@
       <c r="O10" s="7">
         <v>8.8999999999999999E-3</v>
       </c>
-      <c r="P10" s="93">
+      <c r="P10" s="82">
         <v>18.399999999999999</v>
       </c>
-      <c r="Q10" s="91">
+      <c r="Q10" s="80">
         <v>3.26</v>
       </c>
     </row>
     <row r="11" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="110"/>
-      <c r="C11" s="103"/>
-      <c r="D11" s="99"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="85" t="s">
+      <c r="B11" s="93"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="90"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="104" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="86"/>
-      <c r="H11" s="86"/>
-      <c r="I11" s="86"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="86"/>
-      <c r="M11" s="86"/>
-      <c r="N11" s="86"/>
-      <c r="O11" s="87"/>
-      <c r="P11" s="94"/>
-      <c r="Q11" s="92"/>
+      <c r="G11" s="109"/>
+      <c r="H11" s="109"/>
+      <c r="I11" s="109"/>
+      <c r="J11" s="109"/>
+      <c r="K11" s="109"/>
+      <c r="L11" s="109"/>
+      <c r="M11" s="109"/>
+      <c r="N11" s="109"/>
+      <c r="O11" s="106"/>
+      <c r="P11" s="83"/>
+      <c r="Q11" s="81"/>
     </row>
     <row r="12" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="101" t="s">
+      <c r="B12" s="97" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="106" t="s">
+      <c r="C12" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="98">
+      <c r="D12" s="89">
         <v>0.23810000000000001</v>
       </c>
-      <c r="E12" s="91">
+      <c r="E12" s="80">
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="F12" s="11">
@@ -3761,18 +3764,18 @@
       <c r="O12" s="7">
         <v>7.1000000000000004E-3</v>
       </c>
-      <c r="P12" s="93">
+      <c r="P12" s="82">
         <v>3.18</v>
       </c>
-      <c r="Q12" s="91">
+      <c r="Q12" s="80">
         <v>1.7</v>
       </c>
     </row>
     <row r="13" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="101"/>
-      <c r="C13" s="107"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="92"/>
+      <c r="B13" s="97"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="81"/>
       <c r="F13" s="12">
         <v>0.107</v>
       </c>
@@ -3803,18 +3806,18 @@
       <c r="O13" s="9">
         <v>0.17469999999999999</v>
       </c>
-      <c r="P13" s="94"/>
-      <c r="Q13" s="92"/>
+      <c r="P13" s="83"/>
+      <c r="Q13" s="81"/>
     </row>
     <row r="14" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="101"/>
-      <c r="C14" s="102" t="s">
+      <c r="B14" s="97"/>
+      <c r="C14" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="98">
+      <c r="D14" s="89">
         <v>0.29709999999999998</v>
       </c>
-      <c r="E14" s="91">
+      <c r="E14" s="80">
         <v>4.4200000000000003E-2</v>
       </c>
       <c r="F14" s="11">
@@ -3847,18 +3850,18 @@
       <c r="O14" s="7">
         <v>1.52E-2</v>
       </c>
-      <c r="P14" s="93">
+      <c r="P14" s="82">
         <v>16.600000000000001</v>
       </c>
-      <c r="Q14" s="91">
+      <c r="Q14" s="80">
         <v>1.49</v>
       </c>
     </row>
     <row r="15" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="101"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="92"/>
+      <c r="B15" s="97"/>
+      <c r="C15" s="94"/>
+      <c r="D15" s="90"/>
+      <c r="E15" s="81"/>
       <c r="F15" s="12">
         <v>0.1263</v>
       </c>
@@ -3889,18 +3892,18 @@
       <c r="O15" s="9">
         <v>0.1082</v>
       </c>
-      <c r="P15" s="94"/>
-      <c r="Q15" s="92"/>
+      <c r="P15" s="83"/>
+      <c r="Q15" s="81"/>
     </row>
     <row r="16" spans="2:22" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="101"/>
-      <c r="C16" s="105" t="s">
+      <c r="B16" s="97"/>
+      <c r="C16" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="98">
+      <c r="D16" s="89">
         <v>0.25019999999999998</v>
       </c>
-      <c r="E16" s="91">
+      <c r="E16" s="80">
         <v>3.6499999999999998E-2</v>
       </c>
       <c r="F16" s="11">
@@ -3933,19 +3936,19 @@
       <c r="O16" s="7">
         <v>7.3000000000000001E-3</v>
       </c>
-      <c r="P16" s="93">
+      <c r="P16" s="82">
         <v>2.92</v>
       </c>
-      <c r="Q16" s="91">
+      <c r="Q16" s="80">
         <v>1.74</v>
       </c>
       <c r="V16" s="1"/>
     </row>
     <row r="17" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="101"/>
-      <c r="C17" s="105"/>
-      <c r="D17" s="99"/>
-      <c r="E17" s="92"/>
+      <c r="B17" s="97"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="90"/>
+      <c r="E17" s="81"/>
       <c r="F17" s="12">
         <v>0.10680000000000001</v>
       </c>
@@ -3976,18 +3979,18 @@
       <c r="O17" s="9">
         <v>0.18659999999999999</v>
       </c>
-      <c r="P17" s="94"/>
-      <c r="Q17" s="92"/>
+      <c r="P17" s="83"/>
+      <c r="Q17" s="81"/>
     </row>
     <row r="18" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="101"/>
-      <c r="C18" s="104" t="s">
+      <c r="B18" s="97"/>
+      <c r="C18" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="98">
+      <c r="D18" s="89">
         <v>0.24879999999999999</v>
       </c>
-      <c r="E18" s="91">
+      <c r="E18" s="80">
         <v>3.39E-2</v>
       </c>
       <c r="F18" s="11">
@@ -4020,18 +4023,18 @@
       <c r="O18" s="7">
         <v>6.3E-3</v>
       </c>
-      <c r="P18" s="93">
+      <c r="P18" s="82">
         <v>3.12</v>
       </c>
-      <c r="Q18" s="91">
+      <c r="Q18" s="80">
         <v>1.8</v>
       </c>
     </row>
     <row r="19" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="101"/>
-      <c r="C19" s="104"/>
-      <c r="D19" s="99"/>
-      <c r="E19" s="92"/>
+      <c r="B19" s="97"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="90"/>
+      <c r="E19" s="81"/>
       <c r="F19" s="12">
         <v>0.10349999999999999</v>
       </c>
@@ -4062,18 +4065,18 @@
       <c r="O19" s="9">
         <v>0.19500000000000001</v>
       </c>
-      <c r="P19" s="94"/>
-      <c r="Q19" s="92"/>
+      <c r="P19" s="83"/>
+      <c r="Q19" s="81"/>
     </row>
     <row r="20" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="101"/>
-      <c r="C20" s="102" t="s">
+      <c r="B20" s="97"/>
+      <c r="C20" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="98">
+      <c r="D20" s="89">
         <v>0.9909</v>
       </c>
-      <c r="E20" s="91">
+      <c r="E20" s="80">
         <v>3.8699999999999998E-2</v>
       </c>
       <c r="F20" s="11">
@@ -4106,18 +4109,18 @@
       <c r="O20" s="7">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="P20" s="93">
+      <c r="P20" s="82">
         <v>1.37</v>
       </c>
-      <c r="Q20" s="91">
+      <c r="Q20" s="80">
         <v>1.385</v>
       </c>
     </row>
     <row r="21" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="101"/>
-      <c r="C21" s="103"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="92"/>
+      <c r="B21" s="97"/>
+      <c r="C21" s="95"/>
+      <c r="D21" s="90"/>
+      <c r="E21" s="81"/>
       <c r="F21" s="12">
         <v>0.1181</v>
       </c>
@@ -4148,20 +4151,20 @@
       <c r="O21" s="9">
         <v>0.214</v>
       </c>
-      <c r="P21" s="94"/>
-      <c r="Q21" s="92"/>
+      <c r="P21" s="83"/>
+      <c r="Q21" s="81"/>
     </row>
     <row r="22" spans="2:17" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="95" t="s">
+      <c r="B22" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="96" t="s">
+      <c r="C22" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="98">
+      <c r="D22" s="89">
         <v>0.23400000000000001</v>
       </c>
-      <c r="E22" s="91">
+      <c r="E22" s="80">
         <v>3.4299999999999997E-2</v>
       </c>
       <c r="F22" s="11">
@@ -4194,44 +4197,44 @@
       <c r="O22" s="7">
         <v>7.7999999999999996E-3</v>
       </c>
-      <c r="P22" s="93">
+      <c r="P22" s="82">
         <v>19</v>
       </c>
-      <c r="Q22" s="91">
+      <c r="Q22" s="80">
         <v>3.4</v>
       </c>
     </row>
     <row r="23" spans="2:17" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="95"/>
-      <c r="C23" s="96"/>
-      <c r="D23" s="99"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="85" t="s">
+      <c r="B23" s="102"/>
+      <c r="C23" s="86"/>
+      <c r="D23" s="90"/>
+      <c r="E23" s="81"/>
+      <c r="F23" s="104" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="86"/>
-      <c r="H23" s="86"/>
-      <c r="I23" s="86"/>
-      <c r="J23" s="86"/>
-      <c r="K23" s="86"/>
-      <c r="L23" s="86"/>
-      <c r="M23" s="86"/>
-      <c r="N23" s="86"/>
-      <c r="O23" s="87"/>
-      <c r="P23" s="94"/>
-      <c r="Q23" s="92"/>
+      <c r="G23" s="109"/>
+      <c r="H23" s="109"/>
+      <c r="I23" s="109"/>
+      <c r="J23" s="109"/>
+      <c r="K23" s="109"/>
+      <c r="L23" s="109"/>
+      <c r="M23" s="109"/>
+      <c r="N23" s="109"/>
+      <c r="O23" s="106"/>
+      <c r="P23" s="83"/>
+      <c r="Q23" s="81"/>
     </row>
     <row r="24" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="63" t="s">
+      <c r="B24" s="71" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="106" t="s">
+      <c r="C24" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="D24" s="98">
+      <c r="D24" s="89">
         <v>0.2296</v>
       </c>
-      <c r="E24" s="91">
+      <c r="E24" s="80">
         <v>3.6400000000000002E-2</v>
       </c>
       <c r="F24" s="11">
@@ -4264,18 +4267,18 @@
       <c r="O24" s="7">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="P24" s="93">
+      <c r="P24" s="82">
         <v>3.29</v>
       </c>
-      <c r="Q24" s="91">
+      <c r="Q24" s="80">
         <v>1.7</v>
       </c>
     </row>
     <row r="25" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="64"/>
-      <c r="C25" s="107"/>
-      <c r="D25" s="99"/>
-      <c r="E25" s="92"/>
+      <c r="B25" s="72"/>
+      <c r="C25" s="85"/>
+      <c r="D25" s="90"/>
+      <c r="E25" s="81"/>
       <c r="F25" s="12">
         <v>0.1096</v>
       </c>
@@ -4306,18 +4309,18 @@
       <c r="O25" s="9">
         <v>0.17330000000000001</v>
       </c>
-      <c r="P25" s="94"/>
-      <c r="Q25" s="92"/>
+      <c r="P25" s="83"/>
+      <c r="Q25" s="81"/>
     </row>
     <row r="26" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="64"/>
-      <c r="C26" s="105" t="s">
+      <c r="B26" s="72"/>
+      <c r="C26" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="D26" s="98">
+      <c r="D26" s="89">
         <v>0.2399</v>
       </c>
-      <c r="E26" s="91">
+      <c r="E26" s="80">
         <v>3.6499999999999998E-2</v>
       </c>
       <c r="F26" s="11">
@@ -4350,18 +4353,18 @@
       <c r="O26" s="7">
         <v>7.3000000000000001E-3</v>
       </c>
-      <c r="P26" s="93">
+      <c r="P26" s="82">
         <v>3.17</v>
       </c>
-      <c r="Q26" s="91">
+      <c r="Q26" s="80">
         <v>1.72</v>
       </c>
     </row>
     <row r="27" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="113"/>
-      <c r="C27" s="112"/>
-      <c r="D27" s="99"/>
-      <c r="E27" s="92"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="88"/>
+      <c r="D27" s="90"/>
+      <c r="E27" s="81"/>
       <c r="F27" s="12">
         <v>0.1099</v>
       </c>
@@ -4392,16 +4395,16 @@
       <c r="O27" s="9">
         <v>0.184</v>
       </c>
-      <c r="P27" s="94"/>
-      <c r="Q27" s="92"/>
+      <c r="P27" s="83"/>
+      <c r="Q27" s="81"/>
     </row>
     <row r="28" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="28"/>
-      <c r="C28" s="60" t="s">
+      <c r="C28" s="74" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="61"/>
-      <c r="E28" s="62"/>
+      <c r="D28" s="75"/>
+      <c r="E28" s="76"/>
       <c r="F28" s="13">
         <v>0.59499999999999997</v>
       </c>
@@ -4437,11 +4440,11 @@
     </row>
     <row r="29" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="28"/>
-      <c r="C29" s="60" t="s">
+      <c r="C29" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="61"/>
-      <c r="E29" s="62"/>
+      <c r="D29" s="75"/>
+      <c r="E29" s="76"/>
       <c r="F29" s="19">
         <v>0.38504641999999994</v>
       </c>
@@ -4476,11 +4479,11 @@
       <c r="Q29" s="42"/>
     </row>
     <row r="30" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C30" s="53" t="s">
+      <c r="C30" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="D30" s="54"/>
-      <c r="E30" s="55"/>
+      <c r="D30" s="78"/>
+      <c r="E30" s="79"/>
       <c r="F30" s="16">
         <v>0.39357755999999999</v>
       </c>
@@ -4537,52 +4540,22 @@
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="Q26:Q27"/>
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="Q24:Q25"/>
-    <mergeCell ref="P24:P25"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B12:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="F11:O11"/>
+    <mergeCell ref="F23:O23"/>
+    <mergeCell ref="F9:O9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="P16:P17"/>
+    <mergeCell ref="Q16:Q17"/>
+    <mergeCell ref="Q18:Q19"/>
+    <mergeCell ref="P18:P19"/>
+    <mergeCell ref="Q20:Q21"/>
+    <mergeCell ref="P20:P21"/>
+    <mergeCell ref="Q22:Q23"/>
+    <mergeCell ref="P22:P23"/>
+    <mergeCell ref="Q12:Q13"/>
     <mergeCell ref="P12:P13"/>
     <mergeCell ref="Q10:Q11"/>
     <mergeCell ref="P10:P11"/>
@@ -4599,22 +4572,52 @@
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="Q4:Q5"/>
     <mergeCell ref="P4:P5"/>
-    <mergeCell ref="F11:O11"/>
-    <mergeCell ref="F23:O23"/>
-    <mergeCell ref="F9:O9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="P16:P17"/>
-    <mergeCell ref="Q16:Q17"/>
-    <mergeCell ref="Q18:Q19"/>
-    <mergeCell ref="P18:P19"/>
-    <mergeCell ref="Q20:Q21"/>
-    <mergeCell ref="P20:P21"/>
-    <mergeCell ref="Q22:Q23"/>
-    <mergeCell ref="P22:P23"/>
-    <mergeCell ref="Q12:Q13"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B12:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="Q26:Q27"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="Q24:Q25"/>
+    <mergeCell ref="P24:P25"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D27">
     <cfRule type="colorScale" priority="30">
@@ -4640,7 +4643,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4 F6 F8 F10 F12 F14 F16 F18 F20 F22 F24 F26">
+  <conditionalFormatting sqref="F6 F4 F8 F10 F12 F14 F16 F18 F20 F22 F24 F26">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -4652,7 +4655,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5 F7 F9 F11 F13 F15 F17 F19 F21 F23 F25 F27">
+  <conditionalFormatting sqref="F7 F5 F9 F11 F13 F15 F17 F19 F21 F23 F25 F27">
     <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
@@ -4664,7 +4667,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5 F7 F13 F15 F17 F19 F21 F25 F27">
+  <conditionalFormatting sqref="F7 F5 F13 F15 F17 F19 F21 F25 F27">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -4676,7 +4679,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4 G6 G8 G10 G12 G14 G16 G18 G20 G22 G24 G26">
+  <conditionalFormatting sqref="G5 G7 G13 G15 G17 G19 G21 G25 G27">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6 G4 G8 G10 G12 G14 G16 G18 G20 G22 G24 G26">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -4688,19 +4703,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G7 G5 G13 G15 G17 G19 G21 G25 G27">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H6 H4 H8 H10 H12 H14 H16 H18 H20 H22 H24 H26">
+  <conditionalFormatting sqref="H4 H6 H8 H10 H12 H14 H16 H18 H20 H22 H24 H26">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -4712,7 +4715,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5 H7 H13 H15 H17 H19 H21 H25 H27">
+  <conditionalFormatting sqref="H7 H5 H13 H15 H17 H19 H21 H25 H27">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -4724,7 +4727,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4 I6 I8 I10 I12 I14 I16 I18 I20 I22 I24 I26">
+  <conditionalFormatting sqref="I5 I7 I13 I15 I17 I19 I21 I25 I27">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6 I4 I8 I10 I12 I14 I16 I18 I20 I22 I24 I26">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -4736,19 +4751,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7 I5 I13 I15 I17 I19 I21 I25 I27">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J6 J4 J8 J10 J12 J14 J16 J18 J20 J22 J24 J26">
+  <conditionalFormatting sqref="J4 J6 J8 J10 J12 J14 J16 J18 J20 J22 J24 J26">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
@@ -4760,7 +4763,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7 J5 J13 J15 J17 J19 J21 J25 J27">
+  <conditionalFormatting sqref="J5 J7 J13 J15 J17 J19 J21 J25 J27">
     <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
@@ -4772,7 +4775,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4 K6 K8 K10 K12 K14 K16 K18 K20 K22 K24 K26">
+  <conditionalFormatting sqref="K6 K4 K8 K10 K12 K14 K16 K18 K20 K22 K24 K26">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -4784,7 +4787,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5 K7 K13 K15 K17 K19 K21 K25 K27">
+  <conditionalFormatting sqref="K7 K5 K13 K15 K17 K19 K21 K25 K27">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -4796,7 +4799,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4 L6 L8 L10 L12 L14 L16 L18 L20 L22 L24 L26">
+  <conditionalFormatting sqref="L6 L4 L8 L10 L12 L14 L16 L18 L20 L22 L24 L26">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -4808,7 +4811,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5 L7 L13 L15 L17 L19 L21 L25 L27">
+  <conditionalFormatting sqref="L7 L5 L13 L15 L17 L19 L21 L25 L27">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -4820,7 +4823,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M4 M6 M8 M10 M12 M14 M16 M18 M20 M22 M24 M26">
+  <conditionalFormatting sqref="M6 M4 M8 M10 M12 M14 M16 M18 M20 M22 M24 M26">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -4832,7 +4835,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5 M7 M13 M15 M17 M19 M21 M25 M27">
+  <conditionalFormatting sqref="M7 M5 M13 M15 M17 M19 M21 M25 M27">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -4844,7 +4847,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6 N4 N8 N10 N12 N14 N16 N18 N20 N22 N24 N26">
+  <conditionalFormatting sqref="N4 N6 N8 N10 N12 N14 N16 N18 N20 N22 N24 N26">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -4856,7 +4859,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5 N7 N13 N15 N17 N19 N21 N25 N27">
+  <conditionalFormatting sqref="N7 N5 N13 N15 N17 N19 N21 N25 N27">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -4868,7 +4871,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O4 O6 O8 O10 O12 O14 O16 O18 O20 O22 O24 O26">
+  <conditionalFormatting sqref="O6 O4 O8 O10 O12 O14 O16 O18 O20 O22 O24 O26">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -4880,7 +4883,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5 O7 O13 O15 O17 O19 O21 O25 O27">
+  <conditionalFormatting sqref="O7 O5 O13 O15 O17 O19 O21 O25 O27">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>